<commit_message>
Refonte des règles : suppression du Juge de Nature et mise en place des manches simultanées
</commit_message>
<xml_diff>
--- a/base_de_données_du_jeu.xlsx
+++ b/base_de_données_du_jeu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yiyang WANG\Desktop\projet_Jeu_de_Cartes_de_Synthese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BA4855-A2BC-4ECF-BBCE-65112DD34522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF418D6-5107-4D8D-B989-4492A76976B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{F88FB99A-B90A-4A2B-898B-B4377796707E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F88FB99A-B90A-4A2B-898B-B4377796707E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -844,7 +844,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -857,17 +857,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -878,7 +869,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -890,32 +887,29 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1235,961 +1229,961 @@
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="18" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="8" t="s">
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="10"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="7"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="7" t="s">
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="6" t="s">
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="16"/>
+      <c r="V2" s="16"/>
+      <c r="W2" s="16"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6" t="s">
+      <c r="E3" s="16"/>
+      <c r="F3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="7" t="s">
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="6" t="s">
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6" t="s">
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="7" t="s">
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="6" t="s">
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="16"/>
+      <c r="W4" s="16"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6" t="s">
+      <c r="E5" s="16"/>
+      <c r="F5" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="7" t="s">
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="6" t="s">
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
-      <c r="V5" s="6"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
       <c r="W5" s="3"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6" t="s">
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="7" t="s">
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="6" t="s">
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="16"/>
       <c r="W6" s="3"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6" t="s">
+      <c r="E7" s="16"/>
+      <c r="F7" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="7" t="s">
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="6" t="s">
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="6"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="6"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
       <c r="W7" s="3"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6" t="s">
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="7" t="s">
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="6" t="s">
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="16"/>
+      <c r="V8" s="16"/>
       <c r="W8" s="3"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="7" t="s">
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="6" t="s">
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="16"/>
+      <c r="U9" s="16"/>
+      <c r="V9" s="16"/>
       <c r="W9" s="3"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="6" t="s">
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6" t="s">
+      <c r="E10" s="16"/>
+      <c r="F10" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="7" t="s">
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="6" t="s">
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
       <c r="W10" s="3"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6" t="s">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6" t="s">
+      <c r="E11" s="16"/>
+      <c r="F11" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="7" t="s">
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="6" t="s">
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="S11" s="16"/>
+      <c r="T11" s="16"/>
+      <c r="U11" s="16"/>
+      <c r="V11" s="16"/>
       <c r="W11" s="3"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6" t="s">
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6" t="s">
+      <c r="E12" s="16"/>
+      <c r="F12" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="7" t="s">
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="6" t="s">
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="16"/>
+      <c r="U12" s="16"/>
+      <c r="V12" s="16"/>
       <c r="W12" s="3"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6" t="s">
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6" t="s">
+      <c r="E13" s="16"/>
+      <c r="F13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="7" t="s">
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="6" t="s">
+      <c r="N13" s="18"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
+      <c r="S13" s="16"/>
+      <c r="T13" s="16"/>
+      <c r="U13" s="16"/>
+      <c r="V13" s="16"/>
       <c r="W13" s="3"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11" t="s">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="7" t="s">
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="6" t="s">
+      <c r="N14" s="18"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="6"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="16"/>
+      <c r="U14" s="16"/>
+      <c r="V14" s="16"/>
       <c r="W14" s="3"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="6" t="s">
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6" t="s">
+      <c r="E15" s="16"/>
+      <c r="F15" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="7" t="s">
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="6" t="s">
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
-      <c r="T15" s="6"/>
-      <c r="U15" s="6"/>
-      <c r="V15" s="6"/>
-      <c r="W15" s="6"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
+      <c r="S15" s="16"/>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="16"/>
+      <c r="W15" s="16"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12" t="s">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="7" t="s">
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="6" t="s">
+      <c r="N16" s="18"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="6"/>
-      <c r="S16" s="6"/>
-      <c r="T16" s="6"/>
-      <c r="U16" s="6"/>
-      <c r="V16" s="6"/>
-      <c r="W16" s="6"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="16"/>
+      <c r="W16" s="16"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5" t="s">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="5"/>
-      <c r="F17" s="6" t="s">
+      <c r="E17" s="19"/>
+      <c r="F17" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="7" t="s">
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="6" t="s">
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="6"/>
-      <c r="T17" s="6"/>
-      <c r="U17" s="6"/>
-      <c r="V17" s="6"/>
-      <c r="W17" s="6"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="16"/>
+      <c r="T17" s="16"/>
+      <c r="U17" s="16"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="16"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6" t="s">
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6" t="s">
+      <c r="E18" s="16"/>
+      <c r="F18" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="7" t="s">
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="6" t="s">
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="6"/>
-      <c r="S18" s="6"/>
-      <c r="T18" s="6"/>
-      <c r="U18" s="6"/>
-      <c r="V18" s="6"/>
-      <c r="W18" s="6"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="16"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6" t="s">
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6" t="s">
+      <c r="E19" s="16"/>
+      <c r="F19" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6" t="s">
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6" t="s">
+      <c r="E20" s="16"/>
+      <c r="F20" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6" t="s">
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6" t="s">
+      <c r="E21" s="16"/>
+      <c r="F21" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="8" t="s">
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="9"/>
-      <c r="T21" s="9"/>
-      <c r="U21" s="9"/>
-      <c r="V21" s="9"/>
-      <c r="W21" s="9"/>
-      <c r="X21" s="10"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="6"/>
+      <c r="W21" s="6"/>
+      <c r="X21" s="7"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6" t="s">
+      <c r="E22" s="16"/>
+      <c r="F22" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="7" t="s">
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="4" t="s">
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="17"/>
+      <c r="U22" s="17"/>
+      <c r="V22" s="17"/>
+      <c r="W22" s="17"/>
+      <c r="X22" s="17"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6" t="s">
+      <c r="E23" s="16"/>
+      <c r="F23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-      <c r="M23" s="7" t="s">
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="6" t="s">
+      <c r="N23" s="18"/>
+      <c r="O23" s="18"/>
+      <c r="P23" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="Q23" s="6"/>
-      <c r="R23" s="6"/>
-      <c r="S23" s="6"/>
-      <c r="T23" s="6"/>
-      <c r="U23" s="6"/>
-      <c r="V23" s="6"/>
-      <c r="W23" s="6"/>
-      <c r="X23" s="6"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="16"/>
+      <c r="T23" s="16"/>
+      <c r="U23" s="16"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="16"/>
+      <c r="X23" s="16"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6" t="s">
+      <c r="E24" s="16"/>
+      <c r="F24" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-      <c r="M24" s="7" t="s">
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
+      <c r="M24" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="6" t="s">
+      <c r="N24" s="18"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
-      <c r="T24" s="6"/>
-      <c r="U24" s="6"/>
-      <c r="V24" s="6"/>
-      <c r="W24" s="6"/>
-      <c r="X24" s="6"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="16"/>
+      <c r="T24" s="16"/>
+      <c r="U24" s="16"/>
+      <c r="V24" s="16"/>
+      <c r="W24" s="16"/>
+      <c r="X24" s="16"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M25" s="7" t="s">
+      <c r="M25" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="N25" s="7"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="6" t="s">
+      <c r="N25" s="18"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="Q25" s="6"/>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
-      <c r="T25" s="6"/>
-      <c r="U25" s="6"/>
-      <c r="V25" s="6"/>
-      <c r="W25" s="6"/>
-      <c r="X25" s="6"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="16"/>
+      <c r="U25" s="16"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="16"/>
+      <c r="X25" s="16"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M26" s="7" t="s">
+      <c r="M26" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="6" t="s">
+      <c r="N26" s="18"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
-      <c r="T26" s="6"/>
-      <c r="U26" s="6"/>
-      <c r="V26" s="6"/>
-      <c r="W26" s="6"/>
-      <c r="X26" s="6"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="16"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="16"/>
+      <c r="W26" s="16"/>
+      <c r="X26" s="16"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M27" s="7" t="s">
+      <c r="M27" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="6" t="s">
+      <c r="N27" s="18"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="Q27" s="6"/>
-      <c r="R27" s="6"/>
-      <c r="S27" s="6"/>
-      <c r="T27" s="6"/>
-      <c r="U27" s="6"/>
-      <c r="V27" s="6"/>
-      <c r="W27" s="6"/>
-      <c r="X27" s="6"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="16"/>
+      <c r="V27" s="16"/>
+      <c r="W27" s="16"/>
+      <c r="X27" s="16"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M28" s="7" t="s">
+      <c r="M28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="6" t="s">
+      <c r="N28" s="18"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
-      <c r="T28" s="6"/>
-      <c r="U28" s="6"/>
-      <c r="V28" s="6"/>
-      <c r="W28" s="6"/>
-      <c r="X28" s="6"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
+      <c r="V28" s="16"/>
+      <c r="W28" s="16"/>
+      <c r="X28" s="16"/>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M29" s="7" t="s">
+      <c r="M29" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="6" t="s">
+      <c r="N29" s="18"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="Q29" s="6"/>
-      <c r="R29" s="6"/>
-      <c r="S29" s="6"/>
-      <c r="T29" s="6"/>
-      <c r="U29" s="6"/>
-      <c r="V29" s="6"/>
-      <c r="W29" s="6"/>
-      <c r="X29" s="6"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="16"/>
+      <c r="T29" s="16"/>
+      <c r="U29" s="16"/>
+      <c r="V29" s="16"/>
+      <c r="W29" s="16"/>
+      <c r="X29" s="16"/>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M30" s="7" t="s">
+      <c r="M30" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="6" t="s">
+      <c r="N30" s="18"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
-      <c r="T30" s="6"/>
-      <c r="U30" s="6"/>
-      <c r="V30" s="6"/>
-      <c r="W30" s="6"/>
-      <c r="X30" s="6"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="16"/>
+      <c r="T30" s="16"/>
+      <c r="U30" s="16"/>
+      <c r="V30" s="16"/>
+      <c r="W30" s="16"/>
+      <c r="X30" s="16"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M31" s="7" t="s">
+      <c r="M31" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="6" t="s">
+      <c r="N31" s="18"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="Q31" s="6"/>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-      <c r="U31" s="6"/>
-      <c r="V31" s="6"/>
-      <c r="W31" s="6"/>
-      <c r="X31" s="6"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="16"/>
+      <c r="T31" s="16"/>
+      <c r="U31" s="16"/>
+      <c r="V31" s="16"/>
+      <c r="W31" s="16"/>
+      <c r="X31" s="16"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M32" s="7" t="s">
+      <c r="M32" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="N32" s="7"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="6" t="s">
+      <c r="N32" s="18"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="Q32" s="6"/>
-      <c r="R32" s="6"/>
-      <c r="S32" s="6"/>
-      <c r="T32" s="6"/>
-      <c r="U32" s="6"/>
-      <c r="V32" s="6"/>
-      <c r="W32" s="6"/>
-      <c r="X32" s="6"/>
+      <c r="Q32" s="16"/>
+      <c r="R32" s="16"/>
+      <c r="S32" s="16"/>
+      <c r="T32" s="16"/>
+      <c r="U32" s="16"/>
+      <c r="V32" s="16"/>
+      <c r="W32" s="16"/>
+      <c r="X32" s="16"/>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M33" s="7" t="s">
+      <c r="M33" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="6" t="s">
+      <c r="N33" s="18"/>
+      <c r="O33" s="18"/>
+      <c r="P33" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="Q33" s="6"/>
-      <c r="R33" s="6"/>
-      <c r="S33" s="6"/>
-      <c r="T33" s="6"/>
-      <c r="U33" s="6"/>
-      <c r="V33" s="6"/>
-      <c r="W33" s="6"/>
-      <c r="X33" s="6"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="S33" s="16"/>
+      <c r="T33" s="16"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="16"/>
+      <c r="W33" s="16"/>
+      <c r="X33" s="16"/>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M34" s="7" t="s">
+      <c r="M34" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="6" t="s">
+      <c r="N34" s="18"/>
+      <c r="O34" s="18"/>
+      <c r="P34" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="Q34" s="6"/>
-      <c r="R34" s="6"/>
-      <c r="S34" s="6"/>
-      <c r="T34" s="6"/>
-      <c r="U34" s="6"/>
-      <c r="V34" s="6"/>
-      <c r="W34" s="6"/>
-      <c r="X34" s="6"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
+      <c r="S34" s="16"/>
+      <c r="T34" s="16"/>
+      <c r="U34" s="16"/>
+      <c r="V34" s="16"/>
+      <c r="W34" s="16"/>
+      <c r="X34" s="16"/>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.3">
       <c r="M35" s="1"/>
@@ -2552,19 +2546,121 @@
       <c r="L58" s="1"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A59" s="16"/>
-      <c r="B59" s="16"/>
-      <c r="C59" s="16"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
+      <c r="A59" s="14"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="10"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10"/>
+      <c r="I59" s="10"/>
+      <c r="J59" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="126">
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:L17"/>
+    <mergeCell ref="M32:O32"/>
+    <mergeCell ref="M33:O33"/>
+    <mergeCell ref="M34:O34"/>
+    <mergeCell ref="P34:X34"/>
+    <mergeCell ref="P22:X22"/>
+    <mergeCell ref="P24:X24"/>
+    <mergeCell ref="P27:X27"/>
+    <mergeCell ref="P25:X25"/>
+    <mergeCell ref="P31:X31"/>
+    <mergeCell ref="P32:X32"/>
+    <mergeCell ref="P33:X33"/>
+    <mergeCell ref="P23:X23"/>
+    <mergeCell ref="P26:X26"/>
+    <mergeCell ref="M30:O30"/>
+    <mergeCell ref="P29:X29"/>
+    <mergeCell ref="P30:X30"/>
+    <mergeCell ref="M31:O31"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:L21"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="P4:W4"/>
+    <mergeCell ref="P15:W15"/>
+    <mergeCell ref="P16:W16"/>
+    <mergeCell ref="P17:W17"/>
+    <mergeCell ref="P18:W18"/>
+    <mergeCell ref="M21:X21"/>
+    <mergeCell ref="M26:O26"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="M27:O27"/>
+    <mergeCell ref="M28:O28"/>
+    <mergeCell ref="P28:X28"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="P6:V6"/>
+    <mergeCell ref="P14:V14"/>
+    <mergeCell ref="P13:V13"/>
+    <mergeCell ref="P10:V10"/>
+    <mergeCell ref="P11:V11"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="P2:W2"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="M7:O7"/>
+    <mergeCell ref="P7:V7"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="P12:V12"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:L11"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="P9:V9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="P8:V8"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="D59:J59"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:L24"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F20:L20"/>
+    <mergeCell ref="F23:L23"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F18:L18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:L15"/>
+    <mergeCell ref="F22:L22"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F8:L8"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:L5"/>
+    <mergeCell ref="F6:L6"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="F10:L10"/>
+    <mergeCell ref="F12:L12"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="F13:L13"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="D4:E4"/>
@@ -2589,108 +2685,6 @@
     <mergeCell ref="M16:O16"/>
     <mergeCell ref="M10:O10"/>
     <mergeCell ref="M11:O11"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F8:L8"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:L5"/>
-    <mergeCell ref="F6:L6"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="F10:L10"/>
-    <mergeCell ref="F12:L12"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="D59:J59"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:L24"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F20:L20"/>
-    <mergeCell ref="F23:L23"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F18:L18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:L19"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:L15"/>
-    <mergeCell ref="F22:L22"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:L14"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:L16"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="P2:W2"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="M7:O7"/>
-    <mergeCell ref="P7:V7"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="P12:V12"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:L11"/>
-    <mergeCell ref="M4:O4"/>
-    <mergeCell ref="P9:V9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="P8:V8"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="P4:W4"/>
-    <mergeCell ref="P15:W15"/>
-    <mergeCell ref="P16:W16"/>
-    <mergeCell ref="P17:W17"/>
-    <mergeCell ref="P18:W18"/>
-    <mergeCell ref="M21:X21"/>
-    <mergeCell ref="M26:O26"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="M27:O27"/>
-    <mergeCell ref="M28:O28"/>
-    <mergeCell ref="P28:X28"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="P5:V5"/>
-    <mergeCell ref="P6:V6"/>
-    <mergeCell ref="P14:V14"/>
-    <mergeCell ref="P13:V13"/>
-    <mergeCell ref="P10:V10"/>
-    <mergeCell ref="P11:V11"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:L17"/>
-    <mergeCell ref="M32:O32"/>
-    <mergeCell ref="M33:O33"/>
-    <mergeCell ref="M34:O34"/>
-    <mergeCell ref="P34:X34"/>
-    <mergeCell ref="P22:X22"/>
-    <mergeCell ref="P24:X24"/>
-    <mergeCell ref="P27:X27"/>
-    <mergeCell ref="P25:X25"/>
-    <mergeCell ref="P31:X31"/>
-    <mergeCell ref="P32:X32"/>
-    <mergeCell ref="P33:X33"/>
-    <mergeCell ref="P23:X23"/>
-    <mergeCell ref="P26:X26"/>
-    <mergeCell ref="M30:O30"/>
-    <mergeCell ref="P29:X29"/>
-    <mergeCell ref="P30:X30"/>
-    <mergeCell ref="M31:O31"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:L21"/>
-    <mergeCell ref="D23:E23"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2700,465 +2694,464 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B38198F-510D-478A-BBAB-8D0A7354A562}">
-  <dimension ref="A1:AK17"/>
+  <dimension ref="A1:AJ14"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18"/>
-      <c r="W1" s="18"/>
-      <c r="X1" s="18"/>
-      <c r="Y1" s="18"/>
-      <c r="Z1" s="18"/>
-      <c r="AA1" s="18"/>
-      <c r="AB1" s="18"/>
-      <c r="AC1" s="18"/>
-      <c r="AD1" s="18"/>
-      <c r="AE1" s="18"/>
-      <c r="AF1" s="18"/>
-      <c r="AG1" s="18"/>
-      <c r="AH1" s="18"/>
-      <c r="AI1" s="18"/>
-      <c r="AJ1" s="18"/>
-    </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
+      <c r="AA1" s="8"/>
+      <c r="AB1" s="8"/>
+      <c r="AC1" s="8"/>
+      <c r="AD1" s="8"/>
+      <c r="AE1" s="8"/>
+      <c r="AF1" s="8"/>
+      <c r="AG1" s="8"/>
+      <c r="AH1" s="8"/>
+      <c r="AI1" s="8"/>
+      <c r="AJ1" s="8"/>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="16" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
-      <c r="W2" s="17"/>
-      <c r="X2" s="17"/>
-      <c r="Y2" s="17"/>
-      <c r="Z2" s="16" t="s">
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="AA2" s="16"/>
-      <c r="AB2" s="16"/>
-      <c r="AC2" s="17"/>
-      <c r="AD2" s="17"/>
-      <c r="AE2" s="17"/>
-      <c r="AF2" s="17"/>
-      <c r="AG2" s="17"/>
-      <c r="AH2" s="17"/>
-      <c r="AI2" s="17"/>
-      <c r="AJ2" s="17"/>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="AA2" s="14"/>
+      <c r="AB2" s="14"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10"/>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="10"/>
+      <c r="AJ2" s="10"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="20" t="s">
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="17" t="s">
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="17" t="s">
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="AA3" s="17"/>
-      <c r="AB3" s="17"/>
-      <c r="AC3" s="17" t="s">
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10"/>
+      <c r="AC3" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="AD3" s="17"/>
-      <c r="AE3" s="17"/>
-      <c r="AF3" s="17"/>
-      <c r="AG3" s="17"/>
-      <c r="AH3" s="17"/>
-      <c r="AI3" s="17"/>
-      <c r="AJ3" s="17"/>
-      <c r="AK3" s="21"/>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+      <c r="AD3" s="10"/>
+      <c r="AE3" s="10"/>
+      <c r="AF3" s="10"/>
+      <c r="AG3" s="10"/>
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="10"/>
+      <c r="AJ3" s="10"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="20" t="s">
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="17" t="s">
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="17"/>
-      <c r="S4" s="17"/>
-      <c r="T4" s="17"/>
-      <c r="U4" s="17"/>
-      <c r="V4" s="17"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="17"/>
-      <c r="Y4" s="17"/>
-      <c r="Z4" s="17" t="s">
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+      <c r="Y4" s="10"/>
+      <c r="Z4" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="AA4" s="17"/>
-      <c r="AB4" s="17"/>
-      <c r="AC4" s="17" t="s">
+      <c r="AA4" s="10"/>
+      <c r="AB4" s="10"/>
+      <c r="AC4" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="AD4" s="17"/>
-      <c r="AE4" s="17"/>
-      <c r="AF4" s="17"/>
-      <c r="AG4" s="17"/>
-      <c r="AH4" s="17"/>
-      <c r="AI4" s="17"/>
-      <c r="AJ4" s="17"/>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="AD4" s="10"/>
+      <c r="AE4" s="10"/>
+      <c r="AF4" s="10"/>
+      <c r="AG4" s="10"/>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="10"/>
+      <c r="AJ4" s="10"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17" t="s">
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17" t="s">
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-      <c r="U5" s="17"/>
-      <c r="V5" s="17"/>
-      <c r="W5" s="17"/>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
-      <c r="Z5" s="17" t="s">
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="AA5" s="17"/>
-      <c r="AB5" s="17"/>
-      <c r="AC5" s="17" t="s">
+      <c r="AA5" s="10"/>
+      <c r="AB5" s="10"/>
+      <c r="AC5" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="AD5" s="17"/>
-      <c r="AE5" s="17"/>
-      <c r="AF5" s="17"/>
-      <c r="AG5" s="17"/>
-      <c r="AH5" s="17"/>
-      <c r="AI5" s="17"/>
-      <c r="AJ5" s="17"/>
-    </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+      <c r="AD5" s="10"/>
+      <c r="AE5" s="10"/>
+      <c r="AF5" s="10"/>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="10"/>
+      <c r="AJ5" s="10"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17" t="s">
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17" t="s">
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17" t="s">
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="17"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="17"/>
-      <c r="U6" s="17"/>
-      <c r="V6" s="17"/>
-      <c r="W6" s="17"/>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="17" t="s">
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="10"/>
+      <c r="Z6" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="AA6" s="17"/>
-      <c r="AB6" s="17"/>
-      <c r="AC6" s="17" t="s">
+      <c r="AA6" s="10"/>
+      <c r="AB6" s="10"/>
+      <c r="AC6" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="AD6" s="17"/>
-      <c r="AE6" s="17"/>
-      <c r="AF6" s="17"/>
-      <c r="AG6" s="17"/>
-      <c r="AH6" s="17"/>
-      <c r="AI6" s="17"/>
-      <c r="AJ6" s="17"/>
-    </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="AD6" s="10"/>
+      <c r="AE6" s="10"/>
+      <c r="AF6" s="10"/>
+      <c r="AG6" s="10"/>
+      <c r="AH6" s="10"/>
+      <c r="AI6" s="10"/>
+      <c r="AJ6" s="10"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="17" t="s">
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17" t="s">
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17" t="s">
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
-      <c r="R7" s="17"/>
-      <c r="S7" s="17"/>
-      <c r="T7" s="17"/>
-      <c r="U7" s="17"/>
-      <c r="V7" s="17"/>
-      <c r="W7" s="17"/>
-      <c r="X7" s="17"/>
-      <c r="Y7" s="17"/>
-      <c r="Z7" s="17"/>
-      <c r="AA7" s="17"/>
-      <c r="AB7" s="17"/>
-      <c r="AC7" s="17"/>
-      <c r="AD7" s="17"/>
-      <c r="AE7" s="17"/>
-      <c r="AF7" s="17"/>
-      <c r="AG7" s="17"/>
-      <c r="AH7" s="17"/>
-      <c r="AI7" s="17"/>
-      <c r="AJ7" s="17"/>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+      <c r="W7" s="10"/>
+      <c r="X7" s="10"/>
+      <c r="Y7" s="10"/>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="10"/>
+      <c r="AB7" s="10"/>
+      <c r="AC7" s="10"/>
+      <c r="AD7" s="10"/>
+      <c r="AE7" s="10"/>
+      <c r="AF7" s="10"/>
+      <c r="AG7" s="10"/>
+      <c r="AH7" s="10"/>
+      <c r="AI7" s="10"/>
+      <c r="AJ7" s="10"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="17" t="s">
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17" t="s">
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17" t="s">
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="17"/>
-      <c r="R8" s="17"/>
-      <c r="S8" s="17"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="17"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="17"/>
-    </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
+      <c r="Y8" s="10"/>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17" t="s">
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17" t="s">
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="17"/>
-      <c r="R9" s="17"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="17"/>
-      <c r="U9" s="17"/>
-      <c r="V9" s="17"/>
-      <c r="W9" s="17"/>
-      <c r="X9" s="17"/>
-      <c r="Y9" s="17"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
+      <c r="Y9" s="10"/>
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17" t="s">
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17" t="s">
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="17" t="s">
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="P10" s="17"/>
-      <c r="Q10" s="17"/>
-      <c r="R10" s="17"/>
-      <c r="S10" s="17"/>
-      <c r="T10" s="17"/>
-      <c r="U10" s="17"/>
-      <c r="V10" s="17"/>
-      <c r="W10" s="17"/>
-      <c r="X10" s="17"/>
-      <c r="Y10" s="17"/>
-      <c r="Z10" s="17"/>
-      <c r="AA10" s="17"/>
-      <c r="AB10" s="17"/>
-      <c r="AC10" s="17"/>
-      <c r="AD10" s="17"/>
-      <c r="AE10" s="17"/>
-      <c r="AF10" s="17"/>
-      <c r="AG10" s="17"/>
-      <c r="AH10" s="17"/>
-      <c r="AI10" s="17"/>
-      <c r="AJ10" s="17"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A11" s="17" t="s">
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="10"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="10"/>
+      <c r="AD10" s="10"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" s="10"/>
+      <c r="AG10" s="10"/>
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="10"/>
+      <c r="AJ10" s="10"/>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="21" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" t="s">
         <v>157</v>
       </c>
       <c r="E11" s="2"/>
@@ -3169,152 +3162,41 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17" t="s">
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="21"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="21"/>
-      <c r="O12" s="21"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="21"/>
-      <c r="S12" s="21"/>
-      <c r="T12" s="21"/>
-      <c r="U12" s="21"/>
-      <c r="V12" s="21"/>
-      <c r="W12" s="21"/>
-      <c r="X12" s="21"/>
-      <c r="Y12" s="21"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="21"/>
-      <c r="O13" s="21"/>
-      <c r="P13" s="21"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="21"/>
-      <c r="S13" s="21"/>
-      <c r="T13" s="21"/>
-      <c r="U13" s="21"/>
-      <c r="V13" s="21"/>
-      <c r="W13" s="21"/>
-      <c r="X13" s="21"/>
-      <c r="Y13" s="21"/>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21"/>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-    </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="AC10:AJ10"/>
-    <mergeCell ref="Z5:AB5"/>
-    <mergeCell ref="AC5:AJ5"/>
-    <mergeCell ref="Z6:AB6"/>
-    <mergeCell ref="AC6:AJ6"/>
-    <mergeCell ref="AC3:AJ3"/>
-    <mergeCell ref="AC7:AJ7"/>
-    <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="AC4:AJ4"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z10:AB10"/>
-    <mergeCell ref="Z7:AB7"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="O6:Y6"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="O8:Y8"/>
-    <mergeCell ref="O9:Y9"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="O10:Y10"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="O5:Y5"/>
-    <mergeCell ref="O3:Y3"/>
-    <mergeCell ref="O4:Y4"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="O7:Y7"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="L4:N4"/>
-    <mergeCell ref="D6:K6"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:K8"/>
-    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A1:AJ1"/>
+    <mergeCell ref="Z2:AB2"/>
+    <mergeCell ref="D2:K2"/>
+    <mergeCell ref="O2:Y2"/>
+    <mergeCell ref="AC2:AJ2"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="D3:K3"/>
     <mergeCell ref="D12:K12"/>
@@ -3330,12 +3212,40 @@
     <mergeCell ref="D7:K7"/>
     <mergeCell ref="D4:K4"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="D6:K6"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:K8"/>
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:AJ1"/>
-    <mergeCell ref="Z2:AB2"/>
-    <mergeCell ref="D2:K2"/>
-    <mergeCell ref="O2:Y2"/>
-    <mergeCell ref="AC2:AJ2"/>
+    <mergeCell ref="O10:Y10"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="O5:Y5"/>
+    <mergeCell ref="O3:Y3"/>
+    <mergeCell ref="O4:Y4"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="O7:Y7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="O6:Y6"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="O8:Y8"/>
+    <mergeCell ref="O9:Y9"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="AC3:AJ3"/>
+    <mergeCell ref="AC7:AJ7"/>
+    <mergeCell ref="Z4:AB4"/>
+    <mergeCell ref="AC4:AJ4"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z7:AB7"/>
+    <mergeCell ref="AC10:AJ10"/>
+    <mergeCell ref="Z5:AB5"/>
+    <mergeCell ref="AC5:AJ5"/>
+    <mergeCell ref="Z6:AB6"/>
+    <mergeCell ref="AC6:AJ6"/>
+    <mergeCell ref="Z10:AB10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3348,274 +3258,273 @@
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="18" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="8" t="s">
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="10"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="7"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="16" t="s">
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="17" t="s">
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="D3" s="17" t="s">
+      <c r="B3" s="10"/>
+      <c r="D3" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17" t="s">
+      <c r="E3" s="10"/>
+      <c r="F3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="D5" s="17" t="s">
+      <c r="B5" s="10"/>
+      <c r="D5" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17" t="s">
+      <c r="E5" s="10"/>
+      <c r="F5" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17" t="s">
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="D7" s="17" t="s">
+      <c r="B7" s="10"/>
+      <c r="D7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17" t="s">
+      <c r="E7" s="10"/>
+      <c r="F7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="D9" s="17" t="s">
+      <c r="B9" s="10"/>
+      <c r="D9" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17" t="s">
+      <c r="E9" s="10"/>
+      <c r="F9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17" t="s">
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12" t="s">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="14"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="13"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17" t="s">
+      <c r="E13" s="10"/>
+      <c r="F13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M15" s="8" t="s">
+      <c r="M15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="10"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="7"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="M16" s="16" t="s">
+      <c r="M16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="19" t="s">
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="19"/>
-      <c r="W16" s="19"/>
-      <c r="X16" s="19"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+      <c r="V16" s="15"/>
+      <c r="W16" s="15"/>
+      <c r="X16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:L1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:L2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:L3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:L5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:L6"/>
+    <mergeCell ref="M15:X15"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="P16:X16"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:L13"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="P2:V2"/>
+    <mergeCell ref="M1:V1"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:L10"/>
+    <mergeCell ref="F4:L4"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D12:L12"/>
     <mergeCell ref="A7:B7"/>
@@ -3625,17 +3534,18 @@
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="F9:L9"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="P2:V2"/>
-    <mergeCell ref="M1:V1"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:L10"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="M15:X15"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="P16:X16"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:L13"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:L5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:L6"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:L1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:L3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>